<commit_message>
pharmskills v2 with multipages
</commit_message>
<xml_diff>
--- a/app_v2/data_v2/data_evidence_v2.xlsx
+++ b/app_v2/data_v2/data_evidence_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanjana/Documents/01_projects/Pharmskills/pharmskills_app_v2/app_v2/data_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6AA3FC-F422-5744-9D9D-EF29E69F5538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A4CFBC-FBB0-2640-9AA3-03A8AD6EC068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-37660" yWindow="-28200" windowWidth="18520" windowHeight="28200" xr2:uid="{67A7F374-70BF-0D43-951C-BB1EA0CD0AE7}"/>
   </bookViews>
@@ -212,9 +212,6 @@
     <t>Hämorrhoiden</t>
   </si>
   <si>
-    <t>Hamamelisblätter-Extrakt; Lidocain; Bismutgallat; Jojobawachs</t>
-  </si>
-  <si>
     <t>lediglich symptomatische Therapie, Behandlung akuter Beschwerden</t>
   </si>
   <si>
@@ -429,6 +426,9 @@
   </si>
   <si>
     <t>BNO 1016; Cineol</t>
+  </si>
+  <si>
+    <t>Hamamelis; Lidocain; Bismutgallat; Jojobawachs</t>
   </si>
 </sst>
 </file>
@@ -831,7 +831,7 @@
   <cols>
     <col min="1" max="1" width="45.1640625" customWidth="1"/>
     <col min="2" max="2" width="23.1640625" customWidth="1"/>
-    <col min="3" max="3" width="15.5" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
     <col min="4" max="4" width="38.6640625" customWidth="1"/>
     <col min="5" max="5" width="23.1640625" customWidth="1"/>
     <col min="6" max="6" width="20.83203125" customWidth="1"/>
@@ -1196,7 +1196,7 @@
         <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D14" t="s">
         <v>27</v>
@@ -1245,581 +1245,581 @@
         <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>58</v>
+        <v>130</v>
       </c>
       <c r="D16" t="s">
         <v>27</v>
       </c>
       <c r="E16" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" t="s">
+        <v>97</v>
+      </c>
+      <c r="G16" t="s">
         <v>59</v>
       </c>
-      <c r="F16" t="s">
+      <c r="H16" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="G16" t="s">
-        <v>60</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="I16" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
         <v>61</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>62</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" t="s">
         <v>63</v>
       </c>
-      <c r="D17" t="s">
-        <v>70</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
+        <v>97</v>
+      </c>
+      <c r="G17" t="s">
         <v>64</v>
       </c>
-      <c r="F17" t="s">
-        <v>98</v>
-      </c>
-      <c r="G17" t="s">
-        <v>65</v>
-      </c>
       <c r="H17" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D18" t="s">
         <v>27</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D19" t="s">
         <v>27</v>
       </c>
       <c r="E19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F19" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B20" t="s">
         <v>68</v>
       </c>
-      <c r="B20" t="s">
-        <v>69</v>
-      </c>
       <c r="C20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E20" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="D21" t="s">
+        <v>69</v>
+      </c>
+      <c r="E21" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21" t="s">
+        <v>97</v>
+      </c>
+      <c r="G21" t="s">
         <v>70</v>
       </c>
-      <c r="E21" t="s">
-        <v>107</v>
-      </c>
-      <c r="F21" t="s">
-        <v>98</v>
-      </c>
-      <c r="G21" t="s">
-        <v>71</v>
-      </c>
       <c r="H21" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B22" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" t="s">
         <v>75</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>76</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
+        <v>97</v>
+      </c>
+      <c r="G22" t="s">
         <v>77</v>
       </c>
-      <c r="F22" t="s">
-        <v>98</v>
-      </c>
-      <c r="G22" t="s">
-        <v>78</v>
-      </c>
       <c r="H22" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" t="s">
         <v>79</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="D23" t="s">
         <v>27</v>
       </c>
       <c r="E23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F23" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B24" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F24" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B25" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F25" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B26" t="s">
+        <v>110</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>112</v>
       </c>
       <c r="D26" t="s">
         <v>27</v>
       </c>
       <c r="E26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F26" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B27" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="D27" t="s">
         <v>26</v>
       </c>
       <c r="E27" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F27" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G27" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B28" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="D28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F28" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F29" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B30" t="s">
         <v>25</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E30" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B31" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C31" s="3" t="s">
-        <v>96</v>
-      </c>
       <c r="D31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F31" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B32" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C32" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D32" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32" t="s">
         <v>116</v>
       </c>
-      <c r="D32" t="s">
-        <v>70</v>
-      </c>
-      <c r="E32" t="s">
-        <v>117</v>
-      </c>
       <c r="F32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B33" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="D33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E33" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F33" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B34" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F34" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G34" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B35" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D35" t="s">
         <v>69</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="E35" t="s">
         <v>121</v>
       </c>
-      <c r="D35" t="s">
-        <v>70</v>
-      </c>
-      <c r="E35" t="s">
-        <v>122</v>
-      </c>
       <c r="F35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G35" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B36" t="s">
         <v>9</v>
@@ -1828,22 +1828,22 @@
         <v>50</v>
       </c>
       <c r="D36" t="s">
+        <v>122</v>
+      </c>
+      <c r="E36" t="s">
         <v>123</v>
       </c>
-      <c r="E36" t="s">
-        <v>124</v>
-      </c>
       <c r="F36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>